<commit_message>
update: Angola country profile
</commit_message>
<xml_diff>
--- a/reports/Angola_1.1_trade_balance_2003-2024.xlsx
+++ b/reports/Angola_1.1_trade_balance_2003-2024.xlsx
@@ -648,40 +648,40 @@
         <v>16</v>
       </c>
       <c r="B5">
-        <v>10598146741.371</v>
+        <v>10616802794.18</v>
       </c>
       <c r="C5">
         <v>10636226534.624</v>
       </c>
       <c r="D5">
-        <v>31844185776.488</v>
+        <v>31764655499.687</v>
       </c>
       <c r="E5">
-        <v>32047774595.969</v>
+        <v>32047620256.578</v>
       </c>
       <c r="F5">
-        <v>21246039035.117</v>
+        <v>21147852705.507</v>
       </c>
       <c r="G5">
-        <v>21449627854.598</v>
+        <v>21430817462.398</v>
       </c>
       <c r="H5">
-        <v>21411548061.345</v>
+        <v>21411393721.954</v>
       </c>
       <c r="I5">
-        <v>42442332517.859</v>
+        <v>42381458293.867</v>
       </c>
       <c r="J5">
-        <v>42645921337.34</v>
+        <v>42664423050.758</v>
       </c>
       <c r="K5">
-        <v>42684001130.593</v>
+        <v>42683846791.202</v>
       </c>
       <c r="L5">
-        <v>0.9964198023491659</v>
+        <v>0.9981738128291298</v>
       </c>
       <c r="M5">
-        <v>0.9936473336433598</v>
+        <v>0.9911704908312835</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -689,40 +689,40 @@
         <v>17</v>
       </c>
       <c r="B6">
-        <v>11094843413</v>
+        <v>14871732466.38</v>
       </c>
       <c r="C6">
         <v>12662439392.449</v>
       </c>
       <c r="D6">
-        <v>44177783071</v>
+        <v>44336895477.605</v>
       </c>
       <c r="E6">
-        <v>41711887538.549</v>
+        <v>41712202541.479</v>
       </c>
       <c r="F6">
-        <v>33082939658</v>
+        <v>29465163011.22501</v>
       </c>
       <c r="G6">
-        <v>30617044125.549</v>
+        <v>26840470075.09901</v>
       </c>
       <c r="H6">
-        <v>29049448146.10001</v>
+        <v>29049763149.03001</v>
       </c>
       <c r="I6">
-        <v>55272626484</v>
+        <v>59208627943.985</v>
       </c>
       <c r="J6">
-        <v>52806730951.549</v>
+        <v>56583935007.859</v>
       </c>
       <c r="K6">
-        <v>54374326930.998</v>
+        <v>54374641933.928</v>
       </c>
       <c r="L6">
-        <v>0.8762011070012461</v>
+        <v>1.174476102546913</v>
       </c>
       <c r="M6">
-        <v>1.059117332682969</v>
+        <v>1.062923863430994</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1020,7 +1020,7 @@
         <v>21549256530.51</v>
       </c>
       <c r="C14">
-        <v>18527877510.654</v>
+        <v>18527628837.387</v>
       </c>
       <c r="D14">
         <v>33924937478.31</v>
@@ -1035,7 +1035,7 @@
         <v>15289203639.278</v>
       </c>
       <c r="H14">
-        <v>18310582659.134</v>
+        <v>18310831332.401</v>
       </c>
       <c r="I14">
         <v>55474194008.82</v>
@@ -1044,10 +1044,10 @@
         <v>58387716700.298</v>
       </c>
       <c r="K14">
-        <v>55366337680.442</v>
+        <v>55366089007.175</v>
       </c>
       <c r="L14">
-        <v>1.163072052808997</v>
+        <v>1.16308766327538</v>
       </c>
       <c r="M14">
         <v>0.9209108448602463</v>
@@ -1099,40 +1099,40 @@
         <v>27</v>
       </c>
       <c r="B16">
-        <v>15462313478.23</v>
+        <v>16175609038.61</v>
       </c>
       <c r="C16">
-        <v>11877237866.805</v>
+        <v>11877243096.701</v>
       </c>
       <c r="D16">
-        <v>34904881109.37</v>
+        <v>41682666317.85</v>
       </c>
       <c r="E16">
-        <v>36709129296.141</v>
+        <v>36710673515.901</v>
       </c>
       <c r="F16">
-        <v>19442567631.14</v>
+        <v>25507057279.24</v>
       </c>
       <c r="G16">
-        <v>21246815817.911</v>
+        <v>20535064477.291</v>
       </c>
       <c r="H16">
-        <v>24831891429.336</v>
+        <v>24833430419.2</v>
       </c>
       <c r="I16">
-        <v>50367194587.60001</v>
+        <v>57858275356.46</v>
       </c>
       <c r="J16">
-        <v>52171442774.371</v>
+        <v>52886282554.511</v>
       </c>
       <c r="K16">
-        <v>48586367162.946</v>
+        <v>48587916612.60201</v>
       </c>
       <c r="L16">
-        <v>1.301844220990532</v>
+        <v>1.361899298255747</v>
       </c>
       <c r="M16">
-        <v>0.9508501503204908</v>
+        <v>1.135437253685782</v>
       </c>
     </row>
     <row r="17" spans="1:13">
@@ -1140,40 +1140,40 @@
         <v>28</v>
       </c>
       <c r="B17">
-        <v>16006910579.064</v>
+        <v>16549641599.36</v>
       </c>
       <c r="C17">
-        <v>10350369164.713</v>
+        <v>10350424681.27</v>
       </c>
       <c r="D17">
-        <v>40664718814.96</v>
+        <v>41651716643.361</v>
       </c>
       <c r="E17">
-        <v>44190083954.163</v>
+        <v>44191740663.673</v>
       </c>
       <c r="F17">
-        <v>24657808235.896</v>
+        <v>25102075044.001</v>
       </c>
       <c r="G17">
-        <v>28183173375.099</v>
+        <v>27642099064.313</v>
       </c>
       <c r="H17">
-        <v>33839714789.45</v>
+        <v>33841315982.403</v>
       </c>
       <c r="I17">
-        <v>56671629394.024</v>
+        <v>58201358242.721</v>
       </c>
       <c r="J17">
-        <v>60196994533.22701</v>
+        <v>60741382263.033</v>
       </c>
       <c r="K17">
-        <v>54540453118.876</v>
+        <v>54542165344.94299</v>
       </c>
       <c r="L17">
-        <v>1.546506247683954</v>
+        <v>1.598933580890456</v>
       </c>
       <c r="M17">
-        <v>0.9202227100799412</v>
+        <v>0.9425226528268442</v>
       </c>
     </row>
     <row r="18" spans="1:13">
@@ -1181,40 +1181,40 @@
         <v>29</v>
       </c>
       <c r="B18">
-        <v>13961640425.765</v>
+        <v>13967552830.69</v>
       </c>
       <c r="C18">
         <v>9482428808.495001</v>
       </c>
       <c r="D18">
-        <v>35432454858.832</v>
+        <v>35198251385.824</v>
       </c>
       <c r="E18">
-        <v>37513198955.524</v>
+        <v>37514466679.594</v>
       </c>
       <c r="F18">
-        <v>21470814433.067</v>
+        <v>21230698555.134</v>
       </c>
       <c r="G18">
-        <v>23551558529.759</v>
+        <v>23546913848.904</v>
       </c>
       <c r="H18">
-        <v>28030770147.029</v>
+        <v>28032037871.099</v>
       </c>
       <c r="I18">
-        <v>49394095284.597</v>
+        <v>49165804216.514</v>
       </c>
       <c r="J18">
-        <v>51474839381.289</v>
+        <v>51482019510.284</v>
       </c>
       <c r="K18">
-        <v>46995627764.019</v>
+        <v>46996895488.089</v>
       </c>
       <c r="L18">
-        <v>1.472369654202647</v>
+        <v>1.472993165862413</v>
       </c>
       <c r="M18">
-        <v>0.9445330135891916</v>
+        <v>0.9382580775157359</v>
       </c>
     </row>
     <row r="19" spans="1:13">
@@ -1222,40 +1222,40 @@
         <v>30</v>
       </c>
       <c r="B19">
-        <v>9337925708.641001</v>
+        <v>9223139696.639999</v>
       </c>
       <c r="C19">
-        <v>7606312996.74</v>
+        <v>7591876532.368</v>
       </c>
       <c r="D19">
-        <v>22134505473.377</v>
+        <v>22004317640.278</v>
       </c>
       <c r="E19">
-        <v>23953350695.075</v>
+        <v>23910661754.79</v>
       </c>
       <c r="F19">
-        <v>12796579764.736</v>
+        <v>12781177943.638</v>
       </c>
       <c r="G19">
-        <v>14615424986.434</v>
+        <v>14687522058.15</v>
       </c>
       <c r="H19">
-        <v>16347037698.335</v>
+        <v>16318785222.422</v>
       </c>
       <c r="I19">
-        <v>31472431182.018</v>
+        <v>31227457336.918</v>
       </c>
       <c r="J19">
-        <v>33291276403.716</v>
+        <v>33133801451.43</v>
       </c>
       <c r="K19">
-        <v>31559663691.815</v>
+        <v>31502538287.158</v>
       </c>
       <c r="L19">
-        <v>1.227654674826444</v>
+        <v>1.214869559234413</v>
       </c>
       <c r="M19">
-        <v>0.9240671902293832</v>
+        <v>0.9202722143760783</v>
       </c>
     </row>
     <row r="20" spans="1:13">
@@ -1263,40 +1263,40 @@
         <v>31</v>
       </c>
       <c r="B20">
-        <v>11378927920.701</v>
+        <v>11505173904.63</v>
       </c>
       <c r="C20">
-        <v>9438059110.583</v>
+        <v>9450608516.891001</v>
       </c>
       <c r="D20">
-        <v>34472161956.832</v>
+        <v>34984377894.345</v>
       </c>
       <c r="E20">
-        <v>33471591635.577</v>
+        <v>33481373451.457</v>
       </c>
       <c r="F20">
-        <v>23093234036.131</v>
+        <v>23479203989.715</v>
       </c>
       <c r="G20">
-        <v>22092663714.876</v>
+        <v>21976199546.827</v>
       </c>
       <c r="H20">
-        <v>24033532524.994</v>
+        <v>24030764934.56599</v>
       </c>
       <c r="I20">
-        <v>45851089877.533</v>
+        <v>46489551798.975</v>
       </c>
       <c r="J20">
-        <v>44850519556.278</v>
+        <v>44986547356.087</v>
       </c>
       <c r="K20">
-        <v>42909650746.16</v>
+        <v>42931981968.348</v>
       </c>
       <c r="L20">
-        <v>1.205642790257764</v>
+        <v>1.217400327615612</v>
       </c>
       <c r="M20">
-        <v>1.029893120475081</v>
+        <v>1.044890764265305</v>
       </c>
     </row>
     <row r="21" spans="1:13">
@@ -1307,37 +1307,37 @@
         <v>17802935241.948</v>
       </c>
       <c r="C21">
-        <v>14682851945.041</v>
+        <v>14681482987.065</v>
       </c>
       <c r="D21">
         <v>51274951711.647</v>
       </c>
       <c r="E21">
-        <v>53190639478.752</v>
+        <v>53180012707.069</v>
       </c>
       <c r="F21">
         <v>33472016469.699</v>
       </c>
       <c r="G21">
-        <v>35387704236.804</v>
+        <v>35377077465.121</v>
       </c>
       <c r="H21">
-        <v>38507787533.711</v>
+        <v>38498529720.004</v>
       </c>
       <c r="I21">
         <v>69077886953.595</v>
       </c>
       <c r="J21">
-        <v>70993574720.7</v>
+        <v>70982947949.017</v>
       </c>
       <c r="K21">
-        <v>67873491423.793</v>
+        <v>67861495694.134</v>
       </c>
       <c r="L21">
-        <v>1.212498451158243</v>
+        <v>1.212611509180178</v>
       </c>
       <c r="M21">
-        <v>0.9639844945299021</v>
+        <v>0.9641771241027033</v>
       </c>
     </row>
     <row r="22" spans="1:13">
@@ -1345,40 +1345,40 @@
         <v>33</v>
       </c>
       <c r="B22">
-        <v>15695872014.241</v>
+        <v>15572268065.94</v>
       </c>
       <c r="C22">
-        <v>13061790905.181</v>
+        <v>13063347151.473</v>
       </c>
       <c r="D22">
-        <v>39505783208.732</v>
+        <v>38731586575.049</v>
       </c>
       <c r="E22">
-        <v>40149494153.831</v>
+        <v>40157632141.316</v>
       </c>
       <c r="F22">
-        <v>23809911194.491</v>
+        <v>23159318509.109</v>
       </c>
       <c r="G22">
-        <v>24453622139.59</v>
+        <v>24585364075.376</v>
       </c>
       <c r="H22">
-        <v>27087703248.65</v>
+        <v>27094284989.843</v>
       </c>
       <c r="I22">
-        <v>55201655222.973</v>
+        <v>54303854640.98901</v>
       </c>
       <c r="J22">
-        <v>55845366168.072</v>
+        <v>55729900207.256</v>
       </c>
       <c r="K22">
-        <v>53211285059.012</v>
+        <v>53220979292.789</v>
       </c>
       <c r="L22">
-        <v>1.201663089554985</v>
+        <v>1.192058044953976</v>
       </c>
       <c r="M22">
-        <v>0.9839671468180234</v>
+        <v>0.9644888034919814</v>
       </c>
     </row>
     <row r="23" spans="1:13">
@@ -1386,40 +1386,40 @@
         <v>34</v>
       </c>
       <c r="B23">
-        <v>13945978914.08</v>
+        <v>15002678672.72</v>
       </c>
       <c r="C23">
-        <v>12033113299.369</v>
+        <v>12047863821.487</v>
       </c>
       <c r="D23">
-        <v>39250263061.7</v>
+        <v>39371634396.552</v>
       </c>
       <c r="E23">
-        <v>38018109936.056</v>
+        <v>38035265177.61</v>
       </c>
       <c r="F23">
-        <v>25304284147.62</v>
+        <v>24368955723.832</v>
       </c>
       <c r="G23">
-        <v>24072131021.976</v>
+        <v>23032586504.89</v>
       </c>
       <c r="H23">
-        <v>25984996636.687</v>
+        <v>25987401356.123</v>
       </c>
       <c r="I23">
-        <v>53196241975.78</v>
+        <v>54374313069.272</v>
       </c>
       <c r="J23">
-        <v>51964088850.136</v>
+        <v>53037943850.33</v>
       </c>
       <c r="K23">
-        <v>50051223235.425</v>
+        <v>50083128999.097</v>
       </c>
       <c r="L23">
-        <v>1.158966808266594</v>
+        <v>1.2452563288409</v>
       </c>
       <c r="M23">
-        <v>1.032409636557851</v>
+        <v>1.035135004651648</v>
       </c>
     </row>
   </sheetData>

</xml_diff>